<commit_message>
Switch labelling to match my scripts. Maintaining Sara's labelling of radiation as this can easily be changed in my scripts
</commit_message>
<xml_diff>
--- a/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
+++ b/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaan\Documents\#Master Degree\Thesis\Thesis_project\Cell data Sara A549\2025_10_16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80869A44-C848-4906-B2A7-39C7F1F10BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986C5C4D-1A45-4182-A1C0-1CC193681501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="8">
   <si>
-    <t>Radiation</t>
-  </si>
-  <si>
     <t>Experiment</t>
   </si>
   <si>
@@ -39,16 +36,19 @@
     <t>Dose</t>
   </si>
   <si>
-    <t>Flask_number</t>
-  </si>
-  <si>
     <t>Cells plated</t>
   </si>
   <si>
-    <t>Colonies</t>
+    <t>X-ray</t>
   </si>
   <si>
-    <t>X-ray</t>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Rad</t>
+  </si>
+  <si>
+    <t>Triplicate</t>
   </si>
 </sst>
 </file>
@@ -532,8 +532,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
@@ -856,631 +855,307 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="1">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1">
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>500</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="1">
-        <v>2</v>
-      </c>
-      <c r="F3" s="1">
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
         <v>500</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>500</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
         <v>1.7</v>
       </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>1000</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="1">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
         <v>1.7</v>
       </c>
-      <c r="E6" s="1">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1">
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
         <v>1000</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="1">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
         <v>1.7</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7">
         <v>3</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7">
         <v>1000</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1">
-        <v>2</v>
-      </c>
-      <c r="D8" s="1">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
         <v>4.25</v>
       </c>
-      <c r="E8" s="1">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1">
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
         <v>3000</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="1">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
-        <v>2</v>
-      </c>
-      <c r="D9" s="1">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
         <v>4.25</v>
       </c>
-      <c r="E9" s="1">
-        <v>2</v>
-      </c>
-      <c r="F9" s="1">
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
         <v>3000</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9">
         <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1">
-        <v>1</v>
-      </c>
-      <c r="C10" s="1">
-        <v>2</v>
-      </c>
-      <c r="D10" s="1">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
         <v>4.25</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10">
         <v>3</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>3000</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="1">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1">
-        <v>2</v>
-      </c>
-      <c r="D11" s="1">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
         <v>6.8</v>
       </c>
-      <c r="E11" s="1">
-        <v>1</v>
-      </c>
-      <c r="F11" s="1">
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
         <v>6000</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1</v>
-      </c>
-      <c r="C12" s="1">
-        <v>2</v>
-      </c>
-      <c r="D12" s="1">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
         <v>6.8</v>
       </c>
-      <c r="E12" s="1">
-        <v>2</v>
-      </c>
-      <c r="F12" s="1">
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
         <v>6000</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12">
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="1">
-        <v>1</v>
-      </c>
-      <c r="C13" s="1">
-        <v>2</v>
-      </c>
-      <c r="D13" s="1">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
         <v>6.8</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13">
         <v>3</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13">
         <v>6000</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changed the rad labels after all
</commit_message>
<xml_diff>
--- a/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
+++ b/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaan\Documents\#Master Degree\Thesis\Thesis_project\Cell data Sara A549\2025_10_16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986C5C4D-1A45-4182-A1C0-1CC193681501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985071A4-3136-4717-B4F2-AA5ADCAA4282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>Cells plated</t>
   </si>
   <si>
-    <t>X-ray</t>
-  </si>
-  <si>
     <t>Count</t>
   </si>
   <si>
@@ -49,6 +46,9 @@
   </si>
   <si>
     <t>Triplicate</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -860,7 +860,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -872,18 +872,18 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -952,7 +952,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -975,7 +975,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1136,7 +1136,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B13">
         <v>1</v>

</xml_diff>

<commit_message>
Changed X-ray doses to nominal doses
</commit_message>
<xml_diff>
--- a/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
+++ b/Cell data Sara A549/2025_10_16/2025_10_16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhaan\Documents\#Master Degree\Thesis\Thesis_project\Cell data Sara A549\2025_10_16\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985071A4-3136-4717-B4F2-AA5ADCAA4282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9094A4-E357-4EAA-8C51-EEB0E9C5543E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -961,7 +961,7 @@
         <v>2</v>
       </c>
       <c r="D5">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -984,7 +984,7 @@
         <v>2</v>
       </c>
       <c r="D6">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E6">
         <v>2</v>
@@ -1007,7 +1007,7 @@
         <v>2</v>
       </c>
       <c r="D7">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -1030,7 +1030,7 @@
         <v>2</v>
       </c>
       <c r="D8">
-        <v>4.25</v>
+        <v>5</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1053,7 +1053,7 @@
         <v>2</v>
       </c>
       <c r="D9">
-        <v>4.25</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -1076,7 +1076,7 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <v>4.25</v>
+        <v>5</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -1099,7 +1099,7 @@
         <v>2</v>
       </c>
       <c r="D11">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1122,7 +1122,7 @@
         <v>2</v>
       </c>
       <c r="D12">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -1145,7 +1145,7 @@
         <v>2</v>
       </c>
       <c r="D13">
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="E13">
         <v>3</v>

</xml_diff>